<commit_message>
Adjustment to data and study inclusion
</commit_message>
<xml_diff>
--- a/Data/0001-Poeranto_2016.xlsx
+++ b/Data/0001-Poeranto_2016.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/hya21_ic_ac_uk/Documents/PhD/Literature Review/Post-ESA Data Extraction/Extraction/Group Review/GitHubRepo/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2178457135112/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="200" documentId="8_{899C44D9-8A61-415B-97F1-08FDFEAEC230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D69B41E-D7A8-42A7-8C12-3DF2318EB777}"/>
+  <xr:revisionPtr revIDLastSave="201" documentId="8_{899C44D9-8A61-415B-97F1-08FDFEAEC230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FE04DCB-22CE-A643-B77D-D96A321DE782}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{864015B7-DDC4-4993-BEC7-DBFDF8904F8E}"/>
+    <workbookView xWindow="25720" yWindow="840" windowWidth="25240" windowHeight="27700" activeTab="1" xr2:uid="{864015B7-DDC4-4993-BEC7-DBFDF8904F8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Primary" sheetId="1" r:id="rId1"/>
@@ -414,12 +414,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B52BDD8-9B15-4EF0-8606-F39704D45789}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="25.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -433,7 +433,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -447,7 +447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -461,7 +461,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -475,7 +475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -497,12 +497,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7C7FEBC-3DF9-46AB-9086-5A39FE20BD32}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="25.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -516,7 +516,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -530,7 +530,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -544,7 +544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -558,12 +558,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="C5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -580,12 +580,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CE3C464-946C-480B-A0FC-36191CC92258}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -599,7 +599,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -607,17 +607,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>

</xml_diff>